<commit_message>
feat: add Manager Performance Page with tabs for goals, mid-cycle reviews, and end-cycle assessments
- Implemented ManagerPerformancePage component to manage and display performance metrics.
- Added status chips and avatar components for better UI representation.
- Integrated API calls for fetching assignments, mid-cycle reviews, and end-cycle assessments.
- Created skeleton loaders and empty states for improved user experience.
- Developed StatCard and MiniStat components for displaying summary statistics.
- Introduced bulk operations for mid-cycle and end-cycle assessments in the PMS service.
</commit_message>
<xml_diff>
--- a/Backend/Employees-updated.xlsx
+++ b/Backend/Employees-updated.xlsx
@@ -753,7 +753,7 @@
       <c r="K2" s="3" t="n"/>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D46</t>
         </is>
       </c>
       <c r="M2" s="3" t="n"/>
@@ -805,7 +805,7 @@
       <c r="AC2" s="3" t="n"/>
       <c r="AD2" s="3" t="inlineStr">
         <is>
-          <t>DEP005</t>
+          <t>DEP017</t>
         </is>
       </c>
       <c r="AE2" s="3" t="inlineStr">
@@ -863,8 +863,10 @@
           <t>Kaushik.Ramisetty@acronotics.com</t>
         </is>
       </c>
-      <c r="G3" s="4" t="n">
-        <v>9353929971</v>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>9353929971</t>
+        </is>
       </c>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="8" t="n">
@@ -876,7 +878,7 @@
       <c r="K3" s="4" t="n"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D46</t>
         </is>
       </c>
       <c r="M3" s="4" t="n">
@@ -930,7 +932,7 @@
       <c r="AC3" s="4" t="n"/>
       <c r="AD3" s="4" t="inlineStr">
         <is>
-          <t>DEP006</t>
+          <t>DEP017</t>
         </is>
       </c>
       <c r="AE3" s="4" t="inlineStr">
@@ -988,8 +990,10 @@
           <t>Santhoshkumar.N@acronotics.com</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>9480462876</v>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>9480462876</t>
+        </is>
       </c>
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="6" t="n">
@@ -1001,7 +1005,7 @@
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="M4" s="3" t="n"/>
@@ -1051,7 +1055,7 @@
       <c r="AC4" s="3" t="n"/>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>DEP003</t>
+          <t>DEP017</t>
         </is>
       </c>
       <c r="AE4" s="3" t="inlineStr">
@@ -1109,8 +1113,10 @@
           <t>Pranav.j@acronotics.com</t>
         </is>
       </c>
-      <c r="G5" s="4" t="n">
-        <v>8861434569</v>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>8861434569</t>
+        </is>
       </c>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="8" t="n">
@@ -1122,7 +1128,7 @@
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>D17</t>
+          <t>D64</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
@@ -1174,7 +1180,7 @@
       <c r="AC5" s="4" t="n"/>
       <c r="AD5" s="4" t="inlineStr">
         <is>
-          <t>DEP006</t>
+          <t>DEP016</t>
         </is>
       </c>
       <c r="AE5" s="4" t="inlineStr">
@@ -1232,8 +1238,10 @@
           <t>Aashi.Garg@acronotics.com</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>8607151977</v>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>8607151977</t>
+        </is>
       </c>
       <c r="H6" s="3" t="n">
         <v>9620708669</v>
@@ -1247,7 +1255,7 @@
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>D17</t>
+          <t>D46</t>
         </is>
       </c>
       <c r="M6" s="3" t="n"/>
@@ -1299,7 +1307,7 @@
       <c r="AC6" s="3" t="n"/>
       <c r="AD6" s="3" t="inlineStr">
         <is>
-          <t>DEP005</t>
+          <t>DEP017</t>
         </is>
       </c>
       <c r="AE6" s="3" t="inlineStr">
@@ -1374,7 +1382,7 @@
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D64</t>
         </is>
       </c>
       <c r="M7" s="4" t="n"/>
@@ -1426,7 +1434,7 @@
       <c r="AC7" s="4" t="n"/>
       <c r="AD7" s="4" t="inlineStr">
         <is>
-          <t>DEP006</t>
+          <t>DEP016</t>
         </is>
       </c>
       <c r="AE7" s="4" t="inlineStr">
@@ -1436,7 +1444,7 @@
       </c>
       <c r="AF7" s="4" t="inlineStr">
         <is>
-          <t>Pune</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="AG7" s="4" t="inlineStr">

</xml_diff>